<commit_message>
changed the testing code for griffiths example 1. added an excel file with manual calculations.
</commit_message>
<xml_diff>
--- a/inputs/slope/griffiths1_CALCS.xlsx
+++ b/inputs/slope/griffiths1_CALCS.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10727"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10817"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/njones/cursor_projects/xslope/inputs/slope/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6803AFE1-A5BD-0245-8EF7-56DFC95CCA65}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3B85FF62-6E0C-CC47-BFA2-BC9FF97BCBE5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="7360" yWindow="4740" windowWidth="28040" windowHeight="17440" xr2:uid="{7F55063B-120D-4B45-8378-C9F43BE4B0AA}"/>
+    <workbookView xWindow="36780" yWindow="7140" windowWidth="28040" windowHeight="17440" xr2:uid="{7F55063B-120D-4B45-8378-C9F43BE4B0AA}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="22">
   <si>
     <t>Sigma1</t>
   </si>
@@ -75,6 +75,33 @@
   </si>
   <si>
     <t>Compression = positive:</t>
+  </si>
+  <si>
+    <t>C_adj</t>
+  </si>
+  <si>
+    <t>phi_adj</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NOTE: The above equations are for when you have sigma1 and sigma2. If you have sigmax and sigmay, you have to do things differently. </t>
+  </si>
+  <si>
+    <t>tau_xy</t>
+  </si>
+  <si>
+    <t>sigma_x</t>
+  </si>
+  <si>
+    <t>sigma_y</t>
+  </si>
+  <si>
+    <t>sig_mean</t>
+  </si>
+  <si>
+    <t>tau_max</t>
+  </si>
+  <si>
+    <t>F:</t>
   </si>
 </sst>
 </file>
@@ -186,13 +213,13 @@
     <xdr:from>
       <xdr:col>5</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>13</xdr:row>
+      <xdr:row>17</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>13</xdr:col>
       <xdr:colOff>127000</xdr:colOff>
-      <xdr:row>18</xdr:row>
+      <xdr:row>22</xdr:row>
       <xdr:rowOff>18143</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -224,6 +251,384 @@
         </a:prstGeom>
       </xdr:spPr>
     </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>199572</xdr:colOff>
+      <xdr:row>28</xdr:row>
+      <xdr:rowOff>27214</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>81643</xdr:colOff>
+      <xdr:row>36</xdr:row>
+      <xdr:rowOff>63500</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="4" name="TextBox 3">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{A6E0ADF5-94FA-3248-0245-BEABDEB157D4}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="1025072" y="5615214"/>
+          <a:ext cx="4835071" cy="1632857"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:schemeClr val="lt1"/>
+        </a:solidFill>
+        <a:ln w="9525" cmpd="sng">
+          <a:solidFill>
+            <a:schemeClr val="lt1">
+              <a:shade val="50000"/>
+            </a:schemeClr>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="0">
+              <a:solidFill>
+                <a:schemeClr val="dk1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t># Yield function from docs/fem/overview.md for compression-positive convention:</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="0">
+              <a:solidFill>
+                <a:schemeClr val="dk1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t># f = (</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="el-GR" sz="1100" b="0">
+              <a:solidFill>
+                <a:schemeClr val="dk1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>σ1 - σ3)/2 - ((σ1 + σ3)/2 * </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="0">
+              <a:solidFill>
+                <a:schemeClr val="dk1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>sin(</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="el-GR" sz="1100" b="0">
+              <a:solidFill>
+                <a:schemeClr val="dk1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>φ) + </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="0">
+              <a:solidFill>
+                <a:schemeClr val="dk1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>c * cos(</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="el-GR" sz="1100" b="0">
+              <a:solidFill>
+                <a:schemeClr val="dk1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>φ))</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:r>
+            <a:rPr lang="el-GR" sz="1100" b="0">
+              <a:solidFill>
+                <a:schemeClr val="dk1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t># </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="0">
+              <a:solidFill>
+                <a:schemeClr val="dk1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>Simplifying: (</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="el-GR" sz="1100" b="0">
+              <a:solidFill>
+                <a:schemeClr val="dk1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>σ1 - σ3)/2 = </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="0">
+              <a:solidFill>
+                <a:schemeClr val="dk1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>tau_max, (</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="el-GR" sz="1100" b="0">
+              <a:solidFill>
+                <a:schemeClr val="dk1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>σ1 + σ3)/2 = </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="0">
+              <a:solidFill>
+                <a:schemeClr val="dk1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>sig_mean</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="0">
+              <a:solidFill>
+                <a:schemeClr val="dk1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t># So: f = tau_max - (sig_mean * sin(</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="el-GR" sz="1100" b="0">
+              <a:solidFill>
+                <a:schemeClr val="dk1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>φ) + </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="0">
+              <a:solidFill>
+                <a:schemeClr val="dk1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>c * cos(</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="el-GR" sz="1100" b="0">
+              <a:solidFill>
+                <a:schemeClr val="dk1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>φ))</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:r>
+            <a:rPr lang="el-GR" sz="1100" b="0">
+              <a:solidFill>
+                <a:schemeClr val="dk1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t># </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="0">
+              <a:solidFill>
+                <a:schemeClr val="dk1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>Yield when f &gt; 0</a:t>
+          </a:r>
+          <a:br>
+            <a:rPr lang="en-US" sz="1100" b="0">
+              <a:solidFill>
+                <a:schemeClr val="dk1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+          </a:br>
+          <a:br>
+            <a:rPr lang="en-US" sz="1100" b="0">
+              <a:solidFill>
+                <a:schemeClr val="dk1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+          </a:br>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="0">
+              <a:solidFill>
+                <a:schemeClr val="dk1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t># Principal stresses (compression positive, tension negative)</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="0">
+              <a:solidFill>
+                <a:schemeClr val="dk1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>sig_mean = (sig_x + sig_y) / 2</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="0">
+              <a:solidFill>
+                <a:schemeClr val="dk1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>tau_max = sqrt(((sig_x - sig_y) / 2)**2 + tau_xy**2)</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:endParaRPr lang="en-US" sz="1100" b="0">
+            <a:solidFill>
+              <a:schemeClr val="dk1"/>
+            </a:solidFill>
+            <a:effectLst/>
+            <a:latin typeface="+mn-lt"/>
+            <a:ea typeface="+mn-ea"/>
+            <a:cs typeface="+mn-cs"/>
+          </a:endParaRPr>
+        </a:p>
+        <a:p>
+          <a:endParaRPr lang="en-US" sz="1100"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
 </xdr:wsDr>
@@ -546,10 +951,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{54D0B998-3203-EA46-96BF-D2A23DE0483B}">
-  <dimension ref="B2:D20"/>
+  <dimension ref="B2:E45"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="2" spans="2:4" x14ac:dyDescent="0.2">
+    <row r="2" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B2" t="s">
         <v>4</v>
       </c>
@@ -560,112 +965,209 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="B4" t="s">
+    <row r="3" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C3">
+        <v>1.3</v>
+      </c>
+    </row>
+    <row r="5" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B5" t="s">
         <v>2</v>
       </c>
-      <c r="C4" s="1">
+      <c r="C5" s="1">
         <v>312.5</v>
       </c>
     </row>
-    <row r="5" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="B5" t="s">
+    <row r="6" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B6" t="s">
+        <v>13</v>
+      </c>
+      <c r="C6" s="1">
+        <f>C5/C3</f>
+        <v>240.38461538461539</v>
+      </c>
+    </row>
+    <row r="7" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B7" t="s">
         <v>3</v>
       </c>
-      <c r="C5">
+      <c r="C7">
         <v>20</v>
       </c>
-      <c r="D5" t="s">
+      <c r="D7" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="6" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="C6">
-        <f>RADIANS(C5)</f>
+    <row r="8" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="C8">
+        <f>RADIANS(C7)</f>
         <v>0.3490658503988659</v>
       </c>
-      <c r="D6" t="s">
+      <c r="D8" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="7" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="B7" t="s">
+    <row r="9" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B9" t="s">
+        <v>14</v>
+      </c>
+      <c r="C9">
+        <f>ATAN(TAN(C8)/C3)</f>
+        <v>0.27298747084039748</v>
+      </c>
+      <c r="E9">
+        <f>DEGREES(C9)</f>
+        <v>15.641029939105405</v>
+      </c>
+    </row>
+    <row r="11" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B11" t="s">
         <v>0</v>
       </c>
-      <c r="C7">
+      <c r="C11">
         <v>-1629.4974583400001</v>
       </c>
     </row>
-    <row r="8" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="B8" t="s">
+    <row r="12" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B12" t="s">
         <v>1</v>
       </c>
-      <c r="C8">
+      <c r="C12">
         <v>-3180.7181048100001</v>
       </c>
     </row>
-    <row r="9" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="B9" t="s">
+    <row r="13" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B13" t="s">
         <v>6</v>
       </c>
-      <c r="C9">
+      <c r="C13">
         <v>59.928785939999997</v>
       </c>
     </row>
-    <row r="11" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="B11" t="s">
+    <row r="15" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B15" t="s">
         <v>7</v>
       </c>
-      <c r="C11">
-        <f>(C7+C8)/2*SIN(C6)-(C7-C8)/2-C4*COS(C6)</f>
-        <v>-1891.8595753985589</v>
-      </c>
-      <c r="D11" t="s">
+      <c r="C15">
+        <f>(C11+C12)/2*SIN(C9)-(C11-C12)/2-C6*COS(C9)</f>
+        <v>-1655.5332921567101</v>
+      </c>
+      <c r="D15" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="12" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="C12">
+    <row r="16" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="C16">
         <v>-1725.21</v>
       </c>
-      <c r="D12" t="s">
+      <c r="D16" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="15" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="B15" t="s">
+    <row r="19" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B19" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="17" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B17" t="s">
+    <row r="21" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B21" t="s">
         <v>0</v>
       </c>
-      <c r="C17">
-        <f>-C8</f>
+      <c r="C21">
         <v>3180.7181048100001</v>
       </c>
-    </row>
-    <row r="18" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B18" t="s">
+      <c r="E21">
+        <f>(C21-C22)/2</f>
+        <v>775.61032323500001</v>
+      </c>
+    </row>
+    <row r="22" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B22" t="s">
         <v>1</v>
       </c>
-      <c r="C18">
-        <f>-C7</f>
+      <c r="C22">
         <v>1629.4974583400001</v>
       </c>
     </row>
-    <row r="20" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B20" t="s">
+    <row r="23" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B23" t="s">
+        <v>6</v>
+      </c>
+      <c r="C23">
+        <v>-59.928785939999997</v>
+      </c>
+    </row>
+    <row r="25" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B25" t="s">
         <v>7</v>
       </c>
-      <c r="C20">
-        <f>(C17-C18)/2-((C17+C18)/2*SIN(C6)+C4*COS(C6))</f>
-        <v>-340.63892892855904</v>
+      <c r="C25">
+        <f>(C21-C22)/2-((C21+C22)/2*SIN(C9)+C6*COS(C9))</f>
+        <v>-104.3126456867102</v>
+      </c>
+    </row>
+    <row r="27" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B27" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="38" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B38" t="s">
+        <v>17</v>
+      </c>
+      <c r="C38">
+        <v>3180.7181048100001</v>
+      </c>
+    </row>
+    <row r="39" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B39" t="s">
+        <v>18</v>
+      </c>
+      <c r="C39">
+        <v>1629.4974583400001</v>
+      </c>
+    </row>
+    <row r="40" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B40" t="s">
+        <v>16</v>
+      </c>
+      <c r="C40">
+        <v>-59.928785939999997</v>
+      </c>
+    </row>
+    <row r="42" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B42" t="s">
+        <v>19</v>
+      </c>
+      <c r="C42">
+        <f>(C38+C39)/2</f>
+        <v>2405.107781575</v>
+      </c>
+    </row>
+    <row r="43" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B43" t="s">
+        <v>20</v>
+      </c>
+      <c r="C43">
+        <f>SQRT(((C38-C39)/2)^2+C40^2)</f>
+        <v>777.92212521109309</v>
+      </c>
+    </row>
+    <row r="45" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B45" t="s">
+        <v>21</v>
+      </c>
+      <c r="C45">
+        <f>C43-(C42*SIN(C9)+C6*COS(C9))</f>
+        <v>-102.00084371061712</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
   <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>